<commit_message>
resultats minsup ESBL 2019-2021 2
</commit_message>
<xml_diff>
--- a/results_minsup_ESBL/minsup_0_001/rep5/summary_cut_off_values0.95.xlsx
+++ b/results_minsup_ESBL/minsup_0_001/rep5/summary_cut_off_values0.95.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve">dataset</t>
   </si>
@@ -26,7 +26,31 @@
     <t xml:space="preserve">2018_BLSE</t>
   </si>
   <si>
+    <t xml:space="preserve">2019_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021_BLSE</t>
+  </si>
+  <si>
     <t xml:space="preserve">2022_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2018_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2019_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2021_non_BLSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2022_non_BLSE</t>
   </si>
 </sst>
 </file>
@@ -382,10 +406,98 @@
         <v>4</v>
       </c>
       <c r="B3" t="n">
-        <v>0.0472219757835958</v>
+        <v>0.0486433029788816</v>
       </c>
       <c r="C3" t="n">
-        <v>1.42056802701562</v>
+        <v>1.41346840741717</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0.0459841598186781</v>
+      </c>
+      <c r="C4" t="n">
+        <v>1.43758972270983</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0.0490086027729701</v>
+      </c>
+      <c r="C5" t="n">
+        <v>1.43081069157604</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0.0474817831315533</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.4069557392334</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0.0298833918731148</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.05612861322642</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0.0292991817142436</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.05699979347669</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0.0299529684535655</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.05774943053348</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0.0309555165794082</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.05837958830207</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0.033789707527194</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.05570595446555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>